<commit_message>
Day 13: regenerate stale crm_database_full.xlsx and dashboard
Sentinel found crm_database_full.xlsx and indonesia_outreach_desk.html
still dated 2026-09-24, missing today's entire 8-send batch (row count
coincidentally matched but content was yesterday's - none of today's
sent companies appeared in the "All Prospects" sheet). crm_database.xlsx
alone had been regenerated after the send batch; the other two exports
were skipped. Now current: 146 prospects, 193 contact-form-queue rows,
9 needs-manual-verification rows, all matching live state.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database_full.xlsx
+++ b/data/crm_database_full.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U139"/>
+  <dimension ref="A1:U147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10630,39 +10630,39 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>info@colovore.com</t>
+          <t>audrey.lau.l.p@singhealth.com.sg</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Jeffrey Springborn</t>
+          <t>Audrey Lau</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Group Chief Communications Officer</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Colovore</t>
+          <t>SingHealth (Singapore General Hospital Campus)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://colovore.com</t>
+          <t>https://www.singhealth.com.sg</t>
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>web_research: https://www.datacenterdynamics.com/en/news/colovore-secures-925m-debt-facility-from-blackstone-for-liquid-cooled-data-center-build-out/ — Secured a $925M Blackstone debt facility to build liquid-cooled colocation supporting up to 250kW per rack via direct-to-chip and rear-door cooling, expanding into Reno, Chicago, and Austin</t>
+          <t>web_research: https://www.singhealth.com.sg/news/announcements/supercomputer-for-complex-health-research-at-new-centre</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -10672,16 +10672,28 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L132" t="n">
-        <v>0</v>
-      </c>
-      <c r="M132" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>1a0d65fddfe6c101</t>
+        </is>
+      </c>
       <c r="N132" t="inlineStr"/>
-      <c r="O132" t="inlineStr"/>
-      <c r="P132" t="inlineStr"/>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
       <c r="Q132" t="inlineStr">
         <is>
           <t>none</t>
@@ -10699,39 +10711,35 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>press@nscale.com</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>Nidhi Chappell</t>
-        </is>
-      </c>
+          <t>help-occ@rp.edu.sg</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr">
         <is>
-          <t>President, AI Infrastructure</t>
+          <t>Office of Corporate Communications</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Nscale</t>
+          <t>Republic Polytechnic (RP) - AI Technology Centre (AITC)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>https://nscale.com</t>
+          <t>https://www.rp.edu.sg</t>
         </is>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>web_research: https://www.prnewswire.com/news-releases/whitefiber-and-nscale-announce-10-year-40-mw-colocation-agreement-representing-approximately-865-million-in-total-contract-value-at-nc-1-ai-data-center-campus-302646399.html — Anchor tenant taking 40MW of critical IT load at WhiteFiber's 150kW/cabinet NC-1 campus (~$865M contract), alongside its own Stargate Norway project targeting 100,000 GPUs by 2026</t>
+          <t>web_research: https://www.rp.edu.sg/about-us/contact-us/</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -10741,16 +10749,28 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L133" t="n">
-        <v>0</v>
-      </c>
-      <c r="M133" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>1a0d65fe2e523eb5</t>
+        </is>
+      </c>
       <c r="N133" t="inlineStr"/>
-      <c r="O133" t="inlineStr"/>
-      <c r="P133" t="inlineStr"/>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
       <c r="Q133" t="inlineStr">
         <is>
           <t>none</t>
@@ -10768,39 +10788,39 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>press@coreweave.com</t>
+          <t>ir@digitalcorereit.com</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Michael Intrator</t>
+          <t>Mabel Tan</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Director, Capital Markets &amp; Investor Relations</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>CoreWeave</t>
+          <t>Digital Core REIT</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>https://coreweave.com</t>
+          <t>https://www.digitalcorereit.com</t>
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>web_research: https://www.businesswire.com/news/home/20250715975958/en/CoreWeave-Announces-Multi-Billion-Dollar-Commitment-to-AI-Infrastructure-in-Pennsylvania — Committing up to $6B to a new AI data center in Lancaster, PA, an initial 100MW facility with potential to expand to 300MW</t>
+          <t>web_research: https://www.digitalcorereit.com/investor-relations/email-alerts-and-ir-contact/default.aspx</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -10810,16 +10830,28 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L134" t="n">
-        <v>0</v>
-      </c>
-      <c r="M134" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>1a0d65fea7d8bcae</t>
+        </is>
+      </c>
       <c r="N134" t="inlineStr"/>
-      <c r="O134" t="inlineStr"/>
-      <c r="P134" t="inlineStr"/>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
       <c r="Q134" t="inlineStr">
         <is>
           <t>none</t>
@@ -10837,27 +10869,35 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>deepinfra@scratchmm.com</t>
+          <t>ir@superx.sg</t>
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Investor Relations</t>
+        </is>
+      </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>DeepInfra</t>
+          <t>SuperX AI Technology Limited</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>https://deepinfra.com</t>
+          <t>https://www.superx.sg</t>
         </is>
       </c>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" t="inlineStr"/>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>web_research: https://www.theglobeandmail.com/investing/markets/markets-news/GlobeNewswire/3184601/deepinfra-expands-ai-inference-capacity-with-first-international-data-center-in-toronto/ — Opened its first international data center, a 1.7MW facility in Toronto housing more than 1,000 NVIDIA Blackwell B300 GPUs for AI inference</t>
+          <t>web_research: https://www.prnewswire.com/news-releases/ai-compute-simplified-st-telemedia-global-data-centres-and-super-x-0cmut4phmwuj.html</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -10867,16 +10907,28 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L135" t="n">
-        <v>0</v>
-      </c>
-      <c r="M135" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>1a0d65fefbbb0c20</t>
+        </is>
+      </c>
       <c r="N135" t="inlineStr"/>
-      <c r="O135" t="inlineStr"/>
-      <c r="P135" t="inlineStr"/>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
       <c r="Q135" t="inlineStr">
         <is>
           <t>none</t>
@@ -10894,39 +10946,39 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>hello@edgemode.io</t>
+          <t>marketing@bitera-dc.com</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Charlie Faulkner</t>
+          <t>Tedy Harjanto</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>EdgeMode Inc.</t>
+          <t>Bitera Data Center (PT Mitra Informatika Gemilang)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://edgemode.io</t>
+          <t>https://www.bitera-dc.com/</t>
         </is>
       </c>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>web_research: https://www.stocktitan.net/news/EDGM/edge-mode-mora-town-council-and-other-developers-of-the-dc-malpica-0l7s578vv02x.html — Presented an estimated EUR3B 'DC Malpica' AI data center campus plan in Mora, Spain -- two 150,000 sqm data centers totaling 300MW -- via its BLACK AI venture with BlackBerry AIF</t>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/bitera-data-center-in-jakarta-indonesia-launches-operations/</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -10936,16 +10988,28 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L136" t="n">
-        <v>0</v>
-      </c>
-      <c r="M136" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>1a0d65fca086c963</t>
+        </is>
+      </c>
       <c r="N136" t="inlineStr"/>
-      <c r="O136" t="inlineStr"/>
-      <c r="P136" t="inlineStr"/>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
       <c r="Q136" t="inlineStr">
         <is>
           <t>none</t>
@@ -10963,39 +11027,35 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>press@edgeconnex.com</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>Don MacNeil</t>
-        </is>
-      </c>
+          <t>media@certisgroup.com</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr"/>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Chief Revenue Officer</t>
+          <t>Media Contact</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>EdgeConneX</t>
+          <t>Certis Group</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://edgeconnex.com</t>
+          <t>https://www.certisgroup.com</t>
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>web_research: https://www.edgeconnex.com/news/press-releases/edgeconnex-and-lambda-to-build-ai-factory-in-chicago-with-industry-leading-high-density-data-center-infrastructure/ — Building 30+MW of high-density data center infrastructure in Chicago and Atlanta for Lambda, combining direct liquid-to-chip and air cooling for AI workloads</t>
+          <t>web_research: https://servers.asus.com/stories/Certis</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -11005,16 +11065,28 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L137" t="n">
-        <v>0</v>
-      </c>
-      <c r="M137" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>1a0d65ff49a422a6</t>
+        </is>
+      </c>
       <c r="N137" t="inlineStr"/>
-      <c r="O137" t="inlineStr"/>
-      <c r="P137" t="inlineStr"/>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
       <c r="Q137" t="inlineStr">
         <is>
           <t>none</t>
@@ -11032,39 +11104,39 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>press@fluidstack.io</t>
+          <t>sales@dtp.net.id</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Gary Wu</t>
+          <t>Michael Alifen</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Director &amp; CEO</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Fluidstack</t>
+          <t>DTP (PT Dwi Tunggal Putra)</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://fluidstack.io</t>
+          <t>https://www.dtp.net.id/</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>web_research: https://investors.terawulf.com/news-events/press-releases/detail/114/terawulf-announces-fluidstack-expansion-with-160-mw-cb-5 — Expanded contracted critical IT load to roughly 360MW at TeraWulf's Lake Mariner HPC campus (adding a new 160MW CB-5 building) to support AI/HPC compute</t>
+          <t>web_research: https://www.dtp.net.id/en/data-center-services/data-center</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -11074,16 +11146,28 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L138" t="n">
-        <v>0</v>
-      </c>
-      <c r="M138" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>1a0d65fd53ad6410</t>
+        </is>
+      </c>
       <c r="N138" t="inlineStr"/>
-      <c r="O138" t="inlineStr"/>
-      <c r="P138" t="inlineStr"/>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
       <c r="Q138" t="inlineStr">
         <is>
           <t>none</t>
@@ -11101,39 +11185,39 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>pr@lambda.ai</t>
+          <t>sales@mettadc.com</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Ken Patchett</t>
+          <t>Sukoco Halim</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>VP of Data Center Infrastructure</t>
+          <t>President Director &amp; CEO</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Lambda, Inc.</t>
+          <t>MettaDC (PT MettaDC Teknologi Indonesia)</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://lambda.ai</t>
+          <t>https://mettadc.com/</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>web_research: https://lambda.ai/blog/lambda-edgeconnex-dc-pr — Building gigawatt-scale 'AI Factories' with a stated target of 3GW of liquid-cooled data center capacity and 1M+ NVIDIA GPUs, including a multibillion-dollar Microsoft infrastructure deal</t>
+          <t>web_research: https://www.theiconomics.com/market-expansion/proyek-pertama-resmi-beroperasi-mettadc-akan-terus-bangun-data-center-hingga-500-mw/</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -11143,16 +11227,28 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L139" t="n">
-        <v>0</v>
-      </c>
-      <c r="M139" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>1a0d65fd1d7dced6</t>
+        </is>
+      </c>
       <c r="N139" t="inlineStr"/>
-      <c r="O139" t="inlineStr"/>
-      <c r="P139" t="inlineStr"/>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
       <c r="Q139" t="inlineStr">
         <is>
           <t>none</t>
@@ -11166,6 +11262,546 @@
       </c>
       <c r="T139" t="inlineStr"/>
       <c r="U139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>info@colovore.com</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Jeffrey Springborn</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Colovore</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>https://colovore.com</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/colovore-secures-925m-debt-facility-from-blackstone-for-liquid-cooled-data-center-build-out/ — Secured a $925M Blackstone debt facility to build liquid-cooled colocation supporting up to 250kW per rack via direct-to-chip and rear-door cooling, expanding into Reno, Chicago, and Austin</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L140" t="n">
+        <v>0</v>
+      </c>
+      <c r="M140" t="inlineStr"/>
+      <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
+      <c r="P140" t="inlineStr"/>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr"/>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr"/>
+      <c r="U140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>press@nscale.com</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Nidhi Chappell</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>President, AI Infrastructure</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Nscale</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>https://nscale.com</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>web_research: https://www.prnewswire.com/news-releases/whitefiber-and-nscale-announce-10-year-40-mw-colocation-agreement-representing-approximately-865-million-in-total-contract-value-at-nc-1-ai-data-center-campus-302646399.html — Anchor tenant taking 40MW of critical IT load at WhiteFiber's 150kW/cabinet NC-1 campus (~$865M contract), alongside its own Stargate Norway project targeting 100,000 GPUs by 2026</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L141" t="n">
+        <v>0</v>
+      </c>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
+      <c r="P141" t="inlineStr"/>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr"/>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr"/>
+      <c r="U141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>press@coreweave.com</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Michael Intrator</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>CoreWeave</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>https://coreweave.com</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>web_research: https://www.businesswire.com/news/home/20250715975958/en/CoreWeave-Announces-Multi-Billion-Dollar-Commitment-to-AI-Infrastructure-in-Pennsylvania — Committing up to $6B to a new AI data center in Lancaster, PA, an initial 100MW facility with potential to expand to 300MW</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L142" t="n">
+        <v>0</v>
+      </c>
+      <c r="M142" t="inlineStr"/>
+      <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr"/>
+      <c r="P142" t="inlineStr"/>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr"/>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr"/>
+      <c r="U142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>deepinfra@scratchmm.com</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr"/>
+      <c r="C143" t="inlineStr"/>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>DeepInfra</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>https://deepinfra.com</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>web_research: https://www.theglobeandmail.com/investing/markets/markets-news/GlobeNewswire/3184601/deepinfra-expands-ai-inference-capacity-with-first-international-data-center-in-toronto/ — Opened its first international data center, a 1.7MW facility in Toronto housing more than 1,000 NVIDIA Blackwell B300 GPUs for AI inference</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L143" t="n">
+        <v>0</v>
+      </c>
+      <c r="M143" t="inlineStr"/>
+      <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr"/>
+      <c r="P143" t="inlineStr"/>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr"/>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr"/>
+      <c r="U143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>hello@edgemode.io</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Charlie Faulkner</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>EdgeMode Inc.</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>https://edgemode.io</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>web_research: https://www.stocktitan.net/news/EDGM/edge-mode-mora-town-council-and-other-developers-of-the-dc-malpica-0l7s578vv02x.html — Presented an estimated EUR3B 'DC Malpica' AI data center campus plan in Mora, Spain -- two 150,000 sqm data centers totaling 300MW -- via its BLACK AI venture with BlackBerry AIF</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L144" t="n">
+        <v>0</v>
+      </c>
+      <c r="M144" t="inlineStr"/>
+      <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
+      <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr"/>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr"/>
+      <c r="U144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>press@edgeconnex.com</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Don MacNeil</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Chief Revenue Officer</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>EdgeConneX</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>https://edgeconnex.com</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>web_research: https://www.edgeconnex.com/news/press-releases/edgeconnex-and-lambda-to-build-ai-factory-in-chicago-with-industry-leading-high-density-data-center-infrastructure/ — Building 30+MW of high-density data center infrastructure in Chicago and Atlanta for Lambda, combining direct liquid-to-chip and air cooling for AI workloads</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L145" t="n">
+        <v>0</v>
+      </c>
+      <c r="M145" t="inlineStr"/>
+      <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
+      <c r="P145" t="inlineStr"/>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr"/>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr"/>
+      <c r="U145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>press@fluidstack.io</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Gary Wu</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Fluidstack</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>https://fluidstack.io</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>web_research: https://investors.terawulf.com/news-events/press-releases/detail/114/terawulf-announces-fluidstack-expansion-with-160-mw-cb-5 — Expanded contracted critical IT load to roughly 360MW at TeraWulf's Lake Mariner HPC campus (adding a new 160MW CB-5 building) to support AI/HPC compute</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L146" t="n">
+        <v>0</v>
+      </c>
+      <c r="M146" t="inlineStr"/>
+      <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
+      <c r="P146" t="inlineStr"/>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr"/>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr"/>
+      <c r="U146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>pr@lambda.ai</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Ken Patchett</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>VP of Data Center Infrastructure</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Lambda, Inc.</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>https://lambda.ai</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>web_research: https://lambda.ai/blog/lambda-edgeconnex-dc-pr — Building gigawatt-scale 'AI Factories' with a stated target of 3GW of liquid-cooled data center capacity and 1M+ NVIDIA GPUs, including a multibillion-dollar Microsoft infrastructure deal</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L147" t="n">
+        <v>0</v>
+      </c>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
+      <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr"/>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr"/>
+      <c r="U147" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11178,7 +11814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L179"/>
+  <dimension ref="A1:L194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19442,7 +20078,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>2026-09-24 Day 12 run: NOT attempted (filled) beyond one confirmation test. This session network egress policy blocks outbound browser CONNECT: confirmed via agentproxy status (recentRelayFailures: connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 and www.singaporetech.edu.sg:443, the latter from a live fill_contact_form() test on this row) and a live fill_contact_form() call against this batch returning navigation_failed: ERR_TUNNEL_CONNECTION_FAILED. Session-wide poli</t>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
@@ -19504,6 +20140,704 @@
       <c r="L179" t="inlineStr">
         <is>
           <t>2026-09-24T02:23:20+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr"/>
+      <c r="B180" t="inlineStr"/>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Bitera Data Center (PT Mitra Informatika Gemilang)</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://www.bitera-dc.com/</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>https://www.bitera-dc.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>20MW Tier III Jakarta colocation facility, ~4,000 racks, ISO 27001 certified.</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>https://www.datacenterdynamics.com/en/news/bitera-data-center-in-jakarta-indonesia-launches-operations/</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:12:28+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr"/>
+      <c r="B181" t="inlineStr"/>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>MettaDC (PT MettaDC Teknologi Indonesia)</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>https://mettadc.com/</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>https://mettadc.com/support</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>35MW Jakarta-area facility live, targeting 500MW total capacity expansion.</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>https://www.theiconomics.com/market-expansion/proyek-pertama-resmi-beroperasi-mettadc-akan-terus-bangun-data-center-hingga-500-mw/</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:12:28+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr"/>
+      <c r="B182" t="inlineStr"/>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>DTP (PT Dwi Tunggal Putra)</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>https://www.dtp.net.id/</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>+62 822-9999-9387</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>+62 21 27096900</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>https://www.dtp.net.id/en/support/customer-care</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Operates 4 Jakarta-area colocation data centers with cold-containment rack rows.</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>https://www.dtp.net.id/en/data-center-services/data-center</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:12:29+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr"/>
+      <c r="B183" t="inlineStr"/>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>K2 Strategic Indonesia (Kuok Group / Sinar Mas Land JV)</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>https://k2strategic.co/indonesia/</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>https://k2strategic.co/contact-us/</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>JV with Sinar Mas Land developing hyperscale data center campuses in Bekasi (K2 JKT1, 58.8MW IT capacity at full build-out, Tier III + LEED Gold) with a second 100MW+ campus planned in Karawang.</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>https://www.datacenterdynamics.com/en/news/kuok-groups-k2-partners-with-sinar-mas-for-jakarta-data-center-campuses/</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:12:29+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr"/>
+      <c r="B184" t="inlineStr"/>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Pure Data Centres (PureDC Jakarta)</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>https://puredc.com/</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>https://puredc.com/contact-us</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Operational 20MW hyperscale facility in the LOGOS Metrolink Logistics Hub, Bekasi/Jakarta (JKT01), 100% renewable-powered, Zero Waste-to-Landfill certified.</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>https://www.datacenterdynamics.com/en/news/pure-dc-launches-data-center-in-jakarta-indonesia/</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:12:29+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr"/>
+      <c r="B185" t="inlineStr"/>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>IDC Indonesia (PT Internetindo Data Centra Indonesia)</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>https://www.idc.co.id/</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>+62 215269988</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>https://www.idc.co.id/</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Indonesia's first carrier-neutral data center operator, now operating 6 facilities across Jakarta, Batam, Bandung, Surabaya and Makassar carrying over 95% of Indonesian internet traffic.</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>https://www.idc.co.id/</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:12:29+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr"/>
+      <c r="B186" t="inlineStr"/>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>SingHealth (Singapore General Hospital Campus)</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>https://www.singhealth.com.sg</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>https://www.singhealth.com.sg/patient-services/contact-us</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>CHROMA supercomputer (NVIDIA DGX A100 systems) deployed at SGH Campus for large-scale medical AI research.</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>https://www.singhealth.com.sg/news/announcements/supercomputer-for-complex-health-research-at-new-centre</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:15:39+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr"/>
+      <c r="B187" t="inlineStr"/>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Digital Core REIT</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>https://www.digitalcorereit.com</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>https://www.digitalcorereit.com/contact-us/default.aspx</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Digital Core REIT's maiden Singapore acquisition, a stake in Digital Loyang 2 data center (Aug 2026).</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>https://www.digitalcorereit.com/investor-relations/email-alerts-and-ir-contact/default.aspx</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:15:39+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr"/>
+      <c r="B188" t="inlineStr"/>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Keppel DC REIT</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>https://www.keppeldcreit.com</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr"/>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>https://www.keppeldcreit.com/en/investor-relations/ir-contact/</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Keppel DC Singapore 9 construction (mid-2026 start), AI-ready Genting Lane campus expansion.</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>https://datacentremagazine.com/news/major-data-centre-operators-awarded-50-mw-each-in-singapore</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:15:39+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr"/>
+      <c r="B189" t="inlineStr"/>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>SuperX AI Technology Limited</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>https://www.superx.sg</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr"/>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>https://www.superx.sg/contact?language=en</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>AI Innovation Centre at STT GDC Singapore 5, NVIDIA Blackwell GPU infrastructure deployment.</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/ai-compute-simplified-st-telemedia-global-data-centres-and-super-x-0cmut4phmwuj.html</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:15:39+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr"/>
+      <c r="B190" t="inlineStr"/>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Certis Group</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>https://www.certisgroup.com</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr"/>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>https://www.certisgroup.com/connect-with-us/</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>800 sqm Centre for Applied Intelligence + ASUS-built data center for AI security operations.</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>https://servers.asus.com/stories/Certis</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:15:39+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr"/>
+      <c r="B191" t="inlineStr"/>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>OVHcloud Singapore</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>https://www.ovhcloud.com</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr"/>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>https://www.ovhcloud.com/en/contact/</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>OVHcloud launched its second Singapore data center (SGP2), described as its most sustainable data centre in Asia Pacific -- no domain-matched personal/generic email found, contact-form only.</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>https://corporate.ovhcloud.com/en/newsroom/ovhcloud-expands-singapore/</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:15:39+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr"/>
+      <c r="B192" t="inlineStr"/>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure Singapore</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/sg/</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/sg/news/media-contacts.html</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Oracle opened a second Oracle Cloud Region in Singapore to meet rapidly growing AI/cloud demand, enabling customers to migrate mission-critical AI workloads -- distinct from the already-queued Oracle Indonesia row; no domain-matched named contact found, contact-form only.</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>https://blogs.oracle.com/cloud-infrastructure/oracle-opens-second-cloud-region-in-singapore</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:15:39+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr"/>
+      <c r="B193" t="inlineStr"/>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>NUS Medicine (Biological Data Center prototype)</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>https://medicine.nus.edu.sg</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr"/>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>https://medicine.nus.edu.sg/contact-us/</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>NUS Medicine, DayOne and Cortical Labs unveiled Singapore's first biological data center prototype (July/Aug 2026): a 20-unit CL1 rack of 16 million living human neurons requiring precise thermal/life-support environmental control, hosted within infrastructure designed and supported by DayOne at the NUS Life Sciences Institute -- distinct entity/facility from the already-covered DayOne row.</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>https://medicine.nus.edu.sg/news/nus-medicine-dayone-and-cortical-labs-unveil-biological-data-center-prototype-in-singapore/</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:15:39+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr"/>
+      <c r="B194" t="inlineStr"/>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>A*STAR Institute of Advanced Intelligence and Computing (IAIC)</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>https://www.a-star.edu.sg/iaic/about-iaic</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr"/>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>https://www.a-star.edu.sg/Contact-Us.aspx</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>2026-09-25 Day 13 run: NOT filled. Confirmed via curl through the agent proxy (recentRelayFailures showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443, a generic control host) and a live fill_contact_form() test against this batch (SingHealth row) which returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint recording the same connect_rejected / 403-to-CONNECT failure for www.singhealth.com.sg:443 moments later. This confir</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>A*STAR formed IAIC (began operations 1 July 2026) by merging the Institute for Infocomm Research (I2R) and Institute of High Performance Computing (IHPC), consolidating AI, HPC/GPU, FPGA, quantum and modelling/simulation compute capabilities under one institute -- no domain-matched named contact found, contact-form only.</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>https://www.frontier-enterprise.com/astar-launches-new-research-institute-to-push-ai-data-and-computing-applications/</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:15:39+00:00</t>
         </is>
       </c>
     </row>
@@ -19518,7 +20852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19875,6 +21209,48 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Renee Goh</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Senior Manager, Investor Relations &amp; Sustainability</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Keppel DC REIT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>renee.goh@keppel.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>web_research: https://www.keppeldcreit.com/en/investor-relations/ir-contact/ — Keppel DC REIT (SGX-listed, separately managed from Keppel Data Centres) owns the Keppel DC Singapore portfolio; Keppel is beginning construction of Keppel DC Singapore 9 in mid-2026 as part of its AI-ready Genting Lane campus expansion, alongside its publicly stated SGP9 floating-data-center seawater-cooling vision.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Email domain (keppel.com) does not match the source/website domain (keppeldcreit.com). Plausible explanation - SGX REIT managers are commonly staffed by the parent corporation and may retain the parent's email domain - but this was not independently confirmed against a first-party page (WebFetch blocked this session), and the campaign applied the same domain-mismatch standard to two other rows this same batch (K2 Strategic, Pure Data Centres), so held to the same bar rather than making an exception.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Day 17: close closer-shape loophole, regenerate stale exports
Sentinel caught that the 09-30 closer-variety fix was gamed rather
than actually fixed: agents avoided the exact flagged "is X already Y,
or still Z" phrase, but 4 of 17 closers still asked a bare "is X
already [settled]?" yes/no question, and 6 of 17 opened with "worth a/
is this worth [X]?" - same underlying shapes, just not the literal
wording that was checked for. Updated email-humanizer-agent.md to
name the lesson explicitly: fix the underlying question structure a
flagged phrase exemplifies, not just that one wording.

Also regenerated crm_database_full.xlsx and the dashboard, both a day
stale (missing today's 17 sends).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database_full.xlsx
+++ b/data/crm_database_full.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U164"/>
+  <dimension ref="A1:U181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12607,39 +12607,39 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>info@colovore.com</t>
+          <t>christina.koh@sttelemediagdc.com</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Jeffrey Springborn</t>
+          <t>Christina Koh</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Head, Group Marketing and Communications</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Colovore</t>
+          <t>ST Telemedia Global Data Centres</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://colovore.com</t>
+          <t>https://www.sttelemediagdc.com</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>web_research: https://www.datacenterdynamics.com/en/news/colovore-secures-925m-debt-facility-from-blackstone-for-liquid-cooled-data-center-build-out/ — Secured a $925M Blackstone debt facility to build liquid-cooled colocation supporting up to 250kW per rack via direct-to-chip and rear-door cooling, expanding into Reno, Chicago, and Austin</t>
+          <t>web_research: https://www.sttelemediagdc.com/newsroom/st-telemedia-global-data-centres-announces-new-executive-appointments — STT GDC operates multiple Singapore data centre campuses and is developing the FutureGrid HVDC-AI testbed; Christina Koh is named alongside Chow Yi as the company's own media contact across its newsroom press releases.</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -12649,16 +12649,28 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L157" t="n">
-        <v>0</v>
-      </c>
-      <c r="M157" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>gmail:1a0f547310677735</t>
+        </is>
+      </c>
       <c r="N157" t="inlineStr"/>
-      <c r="O157" t="inlineStr"/>
-      <c r="P157" t="inlineStr"/>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
       <c r="Q157" t="inlineStr">
         <is>
           <t>none</t>
@@ -12676,39 +12688,35 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>press@nscale.com</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>Nidhi Chappell</t>
-        </is>
-      </c>
+          <t>contactus@synapxe.sg</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr"/>
       <c r="C158" t="inlineStr">
         <is>
-          <t>President, AI Infrastructure</t>
+          <t>General Enquiries</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Nscale</t>
+          <t>Synapxe</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://nscale.com</t>
+          <t>https://www.synapxe.sg</t>
         </is>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>web_research: https://www.prnewswire.com/news-releases/whitefiber-and-nscale-announce-10-year-40-mw-colocation-agreement-representing-approximately-865-million-in-total-contract-value-at-nc-1-ai-data-center-campus-302646399.html — Anchor tenant taking 40MW of critical IT load at WhiteFiber's 150kW/cabinet NC-1 campus (~$865M contract), alongside its own Stargate Norway project targeting 100,000 GPUs by 2026</t>
+          <t>web_research: https://www.synapxe.sg/healthtech/cloud/h-cloud — Synapxe, Singapore's national HealthTech agency, built H-Cloud to rationalise and consolidate local hospital data centres into a modernised, nation-wide private cloud serving all public hospitals, specialty centres, polyclinics and nursing homes.</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
@@ -12718,16 +12726,28 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L158" t="n">
-        <v>0</v>
-      </c>
-      <c r="M158" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5472d8f8548c</t>
+        </is>
+      </c>
       <c r="N158" t="inlineStr"/>
-      <c r="O158" t="inlineStr"/>
-      <c r="P158" t="inlineStr"/>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
       <c r="Q158" t="inlineStr">
         <is>
           <t>none</t>
@@ -12745,39 +12765,35 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>press@coreweave.com</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>Michael Intrator</t>
-        </is>
-      </c>
+          <t>corpcomms@ocbc.com</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr"/>
       <c r="C159" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Group Brand and Communications</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>CoreWeave</t>
+          <t>OCBC Bank</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://coreweave.com</t>
+          <t>https://www.ocbc.com</t>
         </is>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>web_research: https://www.businesswire.com/news/home/20250715975958/en/CoreWeave-Announces-Multi-Billion-Dollar-Commitment-to-AI-Infrastructure-in-Pennsylvania — Committing up to $6B to a new AI data center in Lancaster, PA, an initial 100MW facility with potential to expand to 300MW</t>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/singapores-ocbc-bank-to-introduce-rack-based-data-center-cooling/ — OCBC operates its own S$240M purpose-built data center in Singapore (first purpose-built DC owned by a Singapore bank) and is implementing a rack-based cooling system to cut emissions by 400+ tons/year; separately hiring a Data Centre Facilities Engineer and a Lead, Data Centre Facilities Management (AVP/VP) for the Loyang facility.</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -12787,16 +12803,28 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L159" t="n">
-        <v>0</v>
-      </c>
-      <c r="M159" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5471f98cfb7a</t>
+        </is>
+      </c>
       <c r="N159" t="inlineStr"/>
-      <c r="O159" t="inlineStr"/>
-      <c r="P159" t="inlineStr"/>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
       <c r="Q159" t="inlineStr">
         <is>
           <t>none</t>
@@ -12814,27 +12842,35 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>deepinfra@scratchmm.com</t>
+          <t>investor.relations@keppeldcreit.com</t>
         </is>
       </c>
       <c r="B160" t="inlineStr"/>
-      <c r="C160" t="inlineStr"/>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Investor Relations</t>
+        </is>
+      </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>DeepInfra</t>
+          <t>Keppel DC REIT</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://deepinfra.com</t>
+          <t>https://www.keppeldcreit.com</t>
         </is>
       </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr"/>
-      <c r="H160" t="inlineStr"/>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>web_research: https://www.theglobeandmail.com/investing/markets/markets-news/GlobeNewswire/3184601/deepinfra-expands-ai-inference-capacity-with-first-international-data-center-in-toronto/ — Opened its first international data center, a 1.7MW facility in Toronto housing more than 1,000 NVIDIA Blackwell B300 GPUs for AI inference</t>
+          <t>web_research: https://www.keppeldcreit.com/en/investor-relations/ir-contact/ — Keppel DC REIT is participating in the Keppel DC Singapore 9 build at the AI-ready Genting Lane campus (construction start mid-2026, 19MW), alongside Keppel Data Centre Funds II and III.</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -12844,16 +12880,28 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L160" t="n">
-        <v>0</v>
-      </c>
-      <c r="M160" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54728c833da5</t>
+        </is>
+      </c>
       <c r="N160" t="inlineStr"/>
-      <c r="O160" t="inlineStr"/>
-      <c r="P160" t="inlineStr"/>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
       <c r="Q160" t="inlineStr">
         <is>
           <t>none</t>
@@ -12871,39 +12919,39 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>hello@edgemode.io</t>
+          <t>ir_industrial@mapletree.com.sg</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Charlie Faulkner</t>
+          <t>Cheng Mui Lian</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Investor Relations and Sustainability</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>EdgeMode Inc.</t>
+          <t>Mapletree Industrial Trust</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>https://edgemode.io</t>
+          <t>https://www.mapletreeindustrialtrust.com</t>
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>web_research: https://www.stocktitan.net/news/EDGM/edge-mode-mora-town-council-and-other-developers-of-the-dc-malpica-0l7s578vv02x.html — Presented an estimated EUR3B 'DC Malpica' AI data center campus plan in Mora, Spain -- two 150,000 sqm data centers totaling 300MW -- via its BLACK AI venture with BlackBerry AIF</t>
+          <t>web_research: https://www.mapletreeindustrialtrust.com/about-us/ — Mapletree Industrial Trust's data-centre portfolio is roughly 57% of its S$8.3B total AUM, including the purpose-built 7 Tai Seng Drive facility (fully leased to Equinix Singapore) and the Sunview Drive data centre in Singapore, plus 13 data centres held via JV with Mapletree Investments in North America.</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -12913,16 +12961,28 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L161" t="n">
-        <v>0</v>
-      </c>
-      <c r="M161" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54724a989642</t>
+        </is>
+      </c>
       <c r="N161" t="inlineStr"/>
-      <c r="O161" t="inlineStr"/>
-      <c r="P161" t="inlineStr"/>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
       <c r="Q161" t="inlineStr">
         <is>
           <t>none</t>
@@ -12940,39 +13000,39 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>press@edgeconnex.com</t>
+          <t>lauren.crystal@smc.co</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Don MacNeil</t>
+          <t>Lauren Crystal</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Chief Revenue Officer</t>
+          <t>Head of Communications</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>EdgeConneX</t>
+          <t>Sustainable Metal Cloud (SMC)</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>https://edgeconnex.com</t>
+          <t>https://smc.co</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>web_research: https://www.edgeconnex.com/news/press-releases/edgeconnex-and-lambda-to-build-ai-factory-in-chicago-with-industry-leading-high-density-data-center-infrastructure/ — Building 30+MW of high-density data center infrastructure in Chicago and Atlanta for Lambda, combining direct liquid-to-chip and air cooling for AI workloads</t>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/singapores-sustainable-metal-cloud-outlines-global-expansion-plans/ — Singapore-founded and HQ'd SMC runs fully immersion-cooled NVIDIA GPU clusters (SIN01/SIN02 availability zones at STT GDC) for AI training/inference, achieving a PUE of 1.03 via its HyperCube immersion-cooling technology.</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -12982,16 +13042,28 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L162" t="n">
-        <v>0</v>
-      </c>
-      <c r="M162" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5472318d99a1</t>
+        </is>
+      </c>
       <c r="N162" t="inlineStr"/>
-      <c r="O162" t="inlineStr"/>
-      <c r="P162" t="inlineStr"/>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
       <c r="Q162" t="inlineStr">
         <is>
           <t>none</t>
@@ -13009,39 +13081,39 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>press@fluidstack.io</t>
+          <t>luana.low@gf.com</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Gary Wu</t>
+          <t>Luana Low</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Deputy Director, Corporate Communications (Public Relations, Singapore)</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Fluidstack</t>
+          <t>GlobalFoundries Singapore</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>https://fluidstack.io</t>
+          <t>https://gf.com</t>
         </is>
       </c>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>web_research: https://investors.terawulf.com/news-events/press-releases/detail/114/terawulf-announces-fluidstack-expansion-with-160-mw-cb-5 — Expanded contracted critical IT load to roughly 360MW at TeraWulf's Lake Mariner HPC campus (adding a new 160MW CB-5 building) to support AI/HPC compute</t>
+          <t>web_research: https://www.edb.gov.sg/en/about-edb/media-releases-publications/globalfoundries-opens-us4-billion-expansion-facility-in-singapore.html — GlobalFoundries officially opened a US$4B expansion fab in Singapore (23,000 sqm), its most advanced Singapore semiconductor facility to date, raising overall Singapore capacity to ~1.5M 300mm wafers/year.</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -13051,16 +13123,28 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L163" t="n">
-        <v>0</v>
-      </c>
-      <c r="M163" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>gmail:1a0f547267649121</t>
+        </is>
+      </c>
       <c r="N163" t="inlineStr"/>
-      <c r="O163" t="inlineStr"/>
-      <c r="P163" t="inlineStr"/>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
       <c r="Q163" t="inlineStr">
         <is>
           <t>none</t>
@@ -13078,39 +13162,39 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>pr@lambda.ai</t>
+          <t>nola.pocock@colt.net</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Ken Patchett</t>
+          <t>Nola Pocock</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>VP of Data Center Infrastructure</t>
+          <t>VP, Global Communications (Colt Group)</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Lambda, Inc.</t>
+          <t>Colt Data Centre Services Singapore</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://lambda.ai</t>
+          <t>https://www.coltdatacentres.net</t>
         </is>
       </c>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>web_research: https://lambda.ai/blog/lambda-edgeconnex-dc-pr — Building gigawatt-scale 'AI Factories' with a stated target of 3GW of liquid-cooled data center capacity and 1M+ NVIDIA GPUs, including a multibillion-dollar Microsoft infrastructure deal</t>
+          <t>web_research: https://www.colt.net/resources/insights/connectivity-for-mc-digital-realty-data-centre — Colt operates a Singapore data center at 29A International Business Park Road; Colt Group's own Global Communications lead (covering both Colt Technology Services and Colt Data Centre Services announcements) is Nola Pocock, consistently listed as press contact on colt.net data-centre-related releases.</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -13120,16 +13204,28 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>unsent</t>
+          <t>sent</t>
         </is>
       </c>
       <c r="L164" t="n">
-        <v>0</v>
-      </c>
-      <c r="M164" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5472e0be35ce</t>
+        </is>
+      </c>
       <c r="N164" t="inlineStr"/>
-      <c r="O164" t="inlineStr"/>
-      <c r="P164" t="inlineStr"/>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
       <c r="Q164" t="inlineStr">
         <is>
           <t>none</t>
@@ -13143,6 +13239,1283 @@
       </c>
       <c r="T164" t="inlineStr"/>
       <c r="U164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>tanya.netto@oracle.com</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Tanya Netto</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Communications &amp; PR Lead, ASEAN</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure Singapore</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/sg/</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>web_research: https://blogs.oracle.com/cloud-infrastructure/oracle-opens-second-cloud-region-in-singapore — Oracle opened a second Oracle Cloud Region in Singapore to meet rapidly growing AI/cloud demand, enabling customers to migrate mission-critical AI workloads.</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L165" t="n">
+        <v>1</v>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5472bfb7b7c4</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr"/>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R165" t="inlineStr"/>
+      <c r="S165" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T165" t="inlineStr"/>
+      <c r="U165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>ai.center@binus.edu</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Prof. Bens Pardamean</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Director, Artificial Intelligence R&amp;D Center (AIRDC)</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>BINUS University (AI R&amp;D Center)</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>https://research.binus.ac.id/airdc/</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>+62.21 530 0244</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>web_research: https://research.binus.ac.id/airdc/ ; https://binus.ac.id/2019/04/binus-dirikan-pusat-riset-artificial-intelligence/ — BINUS University AI R&amp;D Center (AIRDC), founded via NVIDIA-BINUS collaboration, operates a GPU cluster for AI research and industry collaboration, directed by Prof. Bens Pardamean</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L166" t="n">
+        <v>1</v>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5475eb87633c</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr"/>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:58+00:00</t>
+        </is>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr"/>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T166" t="inlineStr"/>
+      <c r="U166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>corsec@pancaanugrahwisesa.com</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr"/>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Corporate Secretary</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>PT NexAI Digital Infrastruktur Tbk (MGLV, formerly PT Panca Anugrah Wisesa Tbk)</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>http://pancaanugrahwisesa.com</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>+62 21 718 0349</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>web_research: https://harianenergi.com/detail/1440376/dapat-restu-rupslb-nexai-mantap-garap-bisnis-ai-data-center ; https://bisnisinsight.com/detail/921750/nexai-mglv-resmi-masuk-bisnis-ai-data-center-usai-restu-rupslb — IDX-listed PT NexAI Digital Infrastruktur Tbk (MGLV) received shareholder approval (RUPSLB, July 2026) to formally pivot its core business from furniture/household equipment to AI-based data center infrastructure</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L167" t="n">
+        <v>1</v>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5475ddf337f9</t>
+        </is>
+      </c>
+      <c r="N167" t="inlineStr"/>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:58+00:00</t>
+        </is>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr"/>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T167" t="inlineStr"/>
+      <c r="U167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>info@edgnex.com</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr"/>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>General/Corporate Contact</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>DAMAC Digital (EDGNEX Cikarang AI Campus)</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>https://www.edgnex.com</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>+971 4 373 2 373</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>web_research: https://www.edgnex.com/contact/ ; https://www.idnfinancials.com/news/56071/dubais-damac-digital-to-build-usd-2-3-billion-data-centre-in-cikarang — DAMAC Digital (EDGNEX) is building a $2.3B AI data center in Greenland International Industrial Center, Pasirranji, Bekasi (JKT02/Cikarang AI Campus), designed for high-density AI racks with a projected capacity exceeding 144MW, first phase slated for Q3 2026 completion</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L168" t="n">
+        <v>1</v>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54759960550c</t>
+        </is>
+      </c>
+      <c r="N168" t="inlineStr"/>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R168" t="inlineStr"/>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T168" t="inlineStr"/>
+      <c r="U168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>infodgx@gunadarma.ac.id</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Prof. Dr. Detty Purnamasari</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Head, AI and Robotics Development Team (DGX Development Team)</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Universitas Gunadarma</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>https://www.hpc-hub.gunadarma.ac.id</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>+628-1212-9955-61</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>web_research: https://www.praktikum-hpc.gunadarma.ac.id/kontak/tim-pengembangan-dgx ; https://www.hpc-hub.gunadarma.ac.id/kontak — Prof. Dr. Detty Purnamasari heads the DGX Development Team overseeing Gunadarma University NVIDIA DGX-1 and DGX A100 supercomputers at its dedicated HPC/DGX hub for AI and data-intensive research</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L169" t="n">
+        <v>1</v>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54761cbada73</t>
+        </is>
+      </c>
+      <c r="N169" t="inlineStr"/>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:58+00:00</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R169" t="inlineStr"/>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T169" t="inlineStr"/>
+      <c r="U169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>inquiry@indokeppeldc.com</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr"/>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>General/Corporate Contact</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>IndoData Data Center (Salim Group, formerly IndoKeppel Data Centres)</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>https://indokeppeldc.com</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>+622139520140</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/keppel-salim-group-launch-data-center-in-bogor-indonesia/ ; https://w.media/indokeppel-sees-significant-data-center-opportunities-in-indonesia/ — IndoKeppel Data Centre 1 (IKDC1) in Bogor, a Salim Group/Keppel JV (Salim Group took full ownership in Dec 2025 and relaunched as IndoData Data Center), is a 7-hectare campus planned for 50MW+ of IT power across 3 phases, featuring N+1 water-cooled chillers and dual water supply, with a stated strategic focus on AI and hyperscale computing; IndoData has up to 500MW of power capacity secured under contract with PLN</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L170" t="n">
+        <v>1</v>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5475268bea7a</t>
+        </is>
+      </c>
+      <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R170" t="inlineStr"/>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T170" t="inlineStr"/>
+      <c r="U170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>inquiry@lgsinarmas.com</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr"/>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>General/Corporate Contact</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>LG Sinar Mas Technology Solutions (LG CNS / SM+ JV)</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>https://www.lgsinarmas.com</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>+62-21-31990258</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>web_research: https://www.sinarmas.com/blog/?p=4168 ; https://www.lgsinarmas.com/ — LG Sinar Mas, a joint venture between South Korean DC services provider LG CNS and Sinar Mas-backed PT SMPlus Digital Investment (SM+), is developing a US$300M AI-based data center on a 44,195 sqm facility in Menteng Atas, Setiabudi, Jakarta, scheduled to begin operations in H2 2026</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L171" t="n">
+        <v>1</v>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54756301e30b</t>
+        </is>
+      </c>
+      <c r="N171" t="inlineStr"/>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr"/>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr"/>
+      <c r="U171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>sales@dhs-dc.com</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Stanley Go</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Digital Hyperspace Indonesia (DHI)</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>https://dh-indonesia.com</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>web_research: https://dh-indonesia.com/contact/ ; https://dh-indonesia.com/about/ — PT Digital Hyperspace Indonesia operates DHI, a Tier III hyperscale data center in Pasirranji, Central Cikarang, Bekasi Regency, West Java, with an initial 20MW IT load (1,200,000 SF purpose-built facility), financed by the GTC Fund and co-investors; Operations Manager Stanley Go is ASHRAE BCxP-certified</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L172" t="n">
+        <v>1</v>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>gmail:1a0f547554b25881</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr"/>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr"/>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T172" t="inlineStr"/>
+      <c r="U172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>selena.sheikh@princetondg.com</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Selena Sheikh</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Corporate Communications Associate Director, Public Relations</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Princeton Digital Group (PDG) Indonesia</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>https://princetondg.com</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>web_research: https://princetondg.com/newsroom/princeton-digital-group-launches-its-22mw-hyperscale-data-center-in-greater-jakarta-2/ — PDG operates JC1 (6MW) and JC2 (22MW hyperscale, launched) data centers in Cibitung, Greater Jakarta, and agreed to acquire a 70%% stake in XL Axiata Indonesian data centers (5 sites) with US$100M growth capital committed to expand capacity</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L173" t="n">
+        <v>1</v>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5475a8ba596c</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr"/>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr"/>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T173" t="inlineStr"/>
+      <c r="U173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>info@colovore.com</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Jeffrey Springborn</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Colovore</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>https://colovore.com</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/colovore-secures-925m-debt-facility-from-blackstone-for-liquid-cooled-data-center-build-out/ — Secured a $925M Blackstone debt facility to build liquid-cooled colocation supporting up to 250kW per rack via direct-to-chip and rear-door cooling, expanding into Reno, Chicago, and Austin</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L174" t="n">
+        <v>0</v>
+      </c>
+      <c r="M174" t="inlineStr"/>
+      <c r="N174" t="inlineStr"/>
+      <c r="O174" t="inlineStr"/>
+      <c r="P174" t="inlineStr"/>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr"/>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T174" t="inlineStr"/>
+      <c r="U174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>press@nscale.com</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Nidhi Chappell</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>President, AI Infrastructure</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Nscale</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>https://nscale.com</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>web_research: https://www.prnewswire.com/news-releases/whitefiber-and-nscale-announce-10-year-40-mw-colocation-agreement-representing-approximately-865-million-in-total-contract-value-at-nc-1-ai-data-center-campus-302646399.html — Anchor tenant taking 40MW of critical IT load at WhiteFiber's 150kW/cabinet NC-1 campus (~$865M contract), alongside its own Stargate Norway project targeting 100,000 GPUs by 2026</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L175" t="n">
+        <v>0</v>
+      </c>
+      <c r="M175" t="inlineStr"/>
+      <c r="N175" t="inlineStr"/>
+      <c r="O175" t="inlineStr"/>
+      <c r="P175" t="inlineStr"/>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr"/>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T175" t="inlineStr"/>
+      <c r="U175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>press@coreweave.com</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Michael Intrator</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>CoreWeave</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>https://coreweave.com</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>web_research: https://www.businesswire.com/news/home/20250715975958/en/CoreWeave-Announces-Multi-Billion-Dollar-Commitment-to-AI-Infrastructure-in-Pennsylvania — Committing up to $6B to a new AI data center in Lancaster, PA, an initial 100MW facility with potential to expand to 300MW</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L176" t="n">
+        <v>0</v>
+      </c>
+      <c r="M176" t="inlineStr"/>
+      <c r="N176" t="inlineStr"/>
+      <c r="O176" t="inlineStr"/>
+      <c r="P176" t="inlineStr"/>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr"/>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T176" t="inlineStr"/>
+      <c r="U176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>deepinfra@scratchmm.com</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr"/>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>DeepInfra</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>https://deepinfra.com</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>web_research: https://www.theglobeandmail.com/investing/markets/markets-news/GlobeNewswire/3184601/deepinfra-expands-ai-inference-capacity-with-first-international-data-center-in-toronto/ — Opened its first international data center, a 1.7MW facility in Toronto housing more than 1,000 NVIDIA Blackwell B300 GPUs for AI inference</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L177" t="n">
+        <v>0</v>
+      </c>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
+      <c r="P177" t="inlineStr"/>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr"/>
+      <c r="S177" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T177" t="inlineStr"/>
+      <c r="U177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>hello@edgemode.io</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Charlie Faulkner</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>EdgeMode Inc.</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>https://edgemode.io</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>web_research: https://www.stocktitan.net/news/EDGM/edge-mode-mora-town-council-and-other-developers-of-the-dc-malpica-0l7s578vv02x.html — Presented an estimated EUR3B 'DC Malpica' AI data center campus plan in Mora, Spain -- two 150,000 sqm data centers totaling 300MW -- via its BLACK AI venture with BlackBerry AIF</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L178" t="n">
+        <v>0</v>
+      </c>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
+      <c r="O178" t="inlineStr"/>
+      <c r="P178" t="inlineStr"/>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr"/>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T178" t="inlineStr"/>
+      <c r="U178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>press@edgeconnex.com</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Don MacNeil</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Chief Revenue Officer</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>EdgeConneX</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>https://edgeconnex.com</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>web_research: https://www.edgeconnex.com/news/press-releases/edgeconnex-and-lambda-to-build-ai-factory-in-chicago-with-industry-leading-high-density-data-center-infrastructure/ — Building 30+MW of high-density data center infrastructure in Chicago and Atlanta for Lambda, combining direct liquid-to-chip and air cooling for AI workloads</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L179" t="n">
+        <v>0</v>
+      </c>
+      <c r="M179" t="inlineStr"/>
+      <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr"/>
+      <c r="P179" t="inlineStr"/>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr"/>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T179" t="inlineStr"/>
+      <c r="U179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>press@fluidstack.io</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Gary Wu</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Fluidstack</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>https://fluidstack.io</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>web_research: https://investors.terawulf.com/news-events/press-releases/detail/114/terawulf-announces-fluidstack-expansion-with-160-mw-cb-5 — Expanded contracted critical IT load to roughly 360MW at TeraWulf's Lake Mariner HPC campus (adding a new 160MW CB-5 building) to support AI/HPC compute</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L180" t="n">
+        <v>0</v>
+      </c>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr"/>
+      <c r="O180" t="inlineStr"/>
+      <c r="P180" t="inlineStr"/>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr"/>
+      <c r="S180" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T180" t="inlineStr"/>
+      <c r="U180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>pr@lambda.ai</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Ken Patchett</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>VP of Data Center Infrastructure</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Lambda, Inc.</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>https://lambda.ai</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>web_research: https://lambda.ai/blog/lambda-edgeconnex-dc-pr — Building gigawatt-scale 'AI Factories' with a stated target of 3GW of liquid-cooled data center capacity and 1M+ NVIDIA GPUs, including a multibillion-dollar Microsoft infrastructure deal</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>unsent</t>
+        </is>
+      </c>
+      <c r="L181" t="n">
+        <v>0</v>
+      </c>
+      <c r="M181" t="inlineStr"/>
+      <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr"/>
+      <c r="P181" t="inlineStr"/>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr"/>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T181" t="inlineStr"/>
+      <c r="U181" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13155,7 +14528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L199"/>
+  <dimension ref="A1:L200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13542,10 +14915,14 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>LG CNS's first AI data center build in Indonesia, via JV with Sinar Mas: a ~$300M (Rp4.6T) facility under construction in Jakarta's Kuningan CBD, due 2027; no dedicated contact page/email found</t>
@@ -13630,10 +15007,14 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
           <t>Acquired 240MW of powered land for a new JC4 hyperscale campus in Bekasi (Greater Jakarta), bringing PDG's Indonesia portfolio to 400MW, following groundbreaking on the 120MW AI-ready JC3 campus</t>
@@ -14430,10 +15811,14 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr">
         <is>
           <t>Building a $2.3B, 144MW AI-focused data center in Cikarang, Bekasi (Greenland International Industrial Center) designed for high-density AI racks with a target PUE of 1.32, phase one due for service by December 2026; no independently-verified published business email found, only a contact form</t>
@@ -15532,12 +16917,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Attempted 2026-09-09T07:27Z: browser navigation blocked by this session's network egress policy (confirmed via curl through the agent proxy: CONNECT tunnel failed, response 403; proxy status endpoint recorded connect_rejected / 'gateway answered 403 to CONNECT' for indosatooredoo.com and www.peruri.co.id, confirming a session-wide policy block, not a site-specific issue, consistent with the last 2 batches). Not a code bug - left as pending, needs retry from a session/environment without this res</t>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -16362,12 +17747,12 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Attempted 2026-09-11T07:26:51Z: browser navigation blocked by this session's network egress policy (confirmed via curl through the agent proxy: CONNECT tunnel failed, response 403 for www.morarepublic.co.id:443; proxy status endpoint recorded connect_rejected / 'gateway answered 403 to CONNECT', confirming a session-wide policy block, not a site-specific issue, consistent with prior batches). Not a code bug - left as pending, needs retry from a session/environment without this restriction.</t>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -16558,10 +17943,14 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J72" t="inlineStr">
         <is>
           <t>Pivoted entirely from furniture trading to AI data center services after acquisition by PT Nextier Datamate Center; approved a rights issue of up to 285.7M shares and acquired PT Nextier Askara Center and PT Nextier GenAi Center to build AI data center infrastructure</t>
@@ -17130,12 +18519,12 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Attempted 2026-09-12T07:16:55Z: browser navigation blocked by this session's network egress policy (confirmed via curl through the agent proxy: CONNECT tunnel failed, response 403 for www.ub.ac.id:443 and www.google.com:443; proxy status endpoint recorded connect_rejected / 'gateway answered 403 to CONNECT', confirming a session-wide policy block, not a site-specific issue, consistent with every prior batch). Not a code bug - left as pending, needs retry from a session/environment without this r</t>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -17602,12 +18991,12 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-09-14 dual-channel-backup run: NOT attempted. This session's network egress policy blocked outbound CONNECT (agentproxy status showed repeated connect_rejected / 403-to-CONNECT, e.g. to www.google.com, moments before this batch) -- same root cause documented for Playwright/WebFetch in this environment. No navigation was performed and no fields were filled or guessed. Left as pending for retry in a session where egress isn't blocked.</t>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -18108,10 +19497,14 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
           <t>Keeps sensitive data and AI workloads on-premise (30+ GenAI applications in production) rather than in external cloud, and plans to lift annual technology spending above S$771M under new CEO's AI push</t>
@@ -18766,10 +20159,14 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I120" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J120" t="inlineStr">
         <is>
           <t>Computer Weekly reports Colt built its Jurong East, Singapore facility (SGDC1, Tier 3+) and is introducing new data-centre cooling technology (dry heat exchanges) aiming for a PUE of about 1.3-1.35 -- a direct, publicly stated cooling-efficiency initiative at an active Singapore facility.</t>
@@ -19034,10 +20431,14 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J126" t="inlineStr">
         <is>
           <t>Synapxe, Singapore's national HealthTech agency, built H-Cloud to rationalise and consolidate local hospital data centres into a modernised, nation-wide private cloud serving all public hospitals, specialty centres, polyclinics and nursing homes. No domain-matched named-individual email found, only a contact form.</t>
@@ -19084,10 +20485,14 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J127" t="inlineStr">
         <is>
           <t>Singapore-founded and HQ'd SMC runs fully immersion-cooled NVIDIA GPU clusters (SIN01/SIN02 availability zones at STT GDC) for AI training/inference, with co-CEO Tim Rosenfield stating immersion cooling 'enables high density hosting for GPUs...the sort of hosting we need to see for platforms like [Nvidia's] Grace Blackwell.' No domain-matched published email found (only third-party guessed patterns, not used); routed via contact form.</t>
@@ -19218,10 +20623,14 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J130" t="inlineStr">
         <is>
           <t>GlobalFoundries officially opened its US$4B expansion fab in Singapore (23,000 sqm), its most advanced Singapore semiconductor facility to date, raising overall Singapore capacity to ~1.5M 300mm wafers/year. Named PR contact Luana Low (Public Relations, Singapore) found on GF's own newsroom page, but exact email text was obscured/unrenderable in search results, so not used as a verified address; routed via contact form.</t>
@@ -21000,10 +22409,14 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I169" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J169" t="inlineStr">
         <is>
           <t>Tier III (Uptime Institute) 20MW greenfield hyperscale data center in Cikarang/Jakarta with 2N UPS redundancy and N+1 cooling infrastructure, expandable to 80MW on a 68,000 sqm campus (GTC Fund/China Telecom-backed); Operations Manager Stanley Go holds ASHRAE BCxP (building/mechanical commissioning) credential, a real facilities-engineering signal.</t>
@@ -21894,10 +23307,14 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
       <c r="J188" t="inlineStr">
         <is>
           <t>Keppel DC Singapore 9 construction (mid-2026 start), AI-ready Genting Lane campus expansion.</t>
@@ -22413,6 +23830,60 @@
       <c r="L199" t="inlineStr">
         <is>
           <t>2026-09-30T02:17:08+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Cheng Mui Lian</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Investor Relations and Sustainability</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Mapletree Industrial Trust</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>https://www.mapletreeindustrialtrust.com</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>https://www.mapletreeindustrialtrust.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>2026-10-01 Day 17 run: NOT filled. Confirmed session-wide network egress block before and during this batch: curl via agentproxy status endpoint showed repeated connect_rejected / "gateway answered 403 to CONNECT" for www.google.com:443 (generic control host), and a live fill_contact_form() test against this batch (Mapletree Industrial Trust row, https://www.mapletreeindustrialtrust.com/contact-us/) returned navigation_failed: ERR_TUNNEL_CONNECTION_FAILED, with the proxy status endpoint then rec</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Mapletree Industrial Trust's data-centre portfolio is roughly 57% of its S$8.3B total AUM, including the purpose-built 7 Tai Seng Drive facility (fully leased to Equinix Singapore) and the Sunview Drive data centre in Singapore.</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>https://www.mapletreeindustrialtrust.com/about-us/</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:18:24+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>